<commit_message>
Refactoring the CodeValue, increase Mutation score
</commit_message>
<xml_diff>
--- a/tests/Fixtures/medicines.xlsx
+++ b/tests/Fixtures/medicines.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\work\projects\drudz\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\work\websites\dz-medicines\tests\Fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38A0E0B-BD90-4B27-AC4E-2C74404B2B27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6431B56-2A8B-462D-A48F-7FACE2F339AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nomenclature AOUT 2024" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="182">
   <si>
     <t>REPUBLIQUE ALGERIENNE DEMOCRATIQUE ET POPULAIRE</t>
   </si>
@@ -698,6 +698,9 @@
       </rPr>
       <t>:Les informations détaillées sur le produit pharmaceutique figurent dans la décision enregistrement(DE).</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">    </t>
   </si>
 </sst>
 </file>
@@ -2269,8 +2272,30 @@
         <v>43</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="R28"/>
+    <row r="28" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="12">
+        <v>11</v>
+      </c>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="13"/>
+      <c r="H28" s="13"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="14"/>
+      <c r="L28" s="13"/>
+      <c r="M28" s="13"/>
+      <c r="N28" s="15"/>
+      <c r="O28" s="16"/>
+      <c r="P28" s="16"/>
+      <c r="Q28" s="14"/>
+      <c r="R28" s="17"/>
+      <c r="S28" s="15"/>
     </row>
     <row r="29" spans="1:19" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B29" s="62" t="s">
@@ -3969,6 +3994,7 @@
     <mergeCell ref="A9:R9"/>
     <mergeCell ref="A13:S13"/>
   </mergeCells>
+  <phoneticPr fontId="16" type="noConversion"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="44" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>